<commit_message>
feat: port POQA IT standards; add 2 courses
Lab standards (PKSF/BMET/BWCCI/WEAB Graphic Design, IT Freelancing,
Digital Marketing) take the space row, the full PC/software
configuration and the air-conditioning halving footnote from the
practice-vetted POQA workbook. Item lists and weights kept; the Graphic
"Air-conditioning" row is dropped since the halving rule replaces it.

New courses (162 -> 164):
- BSIA Semiconductor Testing Engineering, 21 items, weights by analogy
  with the other five BSIA sheets (the CS carries none).
- PKSF Housekeeping, a copy of the ISC-T&H standard and CS.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_019iYqT5hGHgxLsLhYPmRGg4
</commit_message>
<xml_diff>
--- a/data/xlsx/bmet--graphic-and-ui-design.xlsx
+++ b/data/xlsx/bmet--graphic-and-ui-design.xlsx
@@ -99,7 +99,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="16">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="bottom"/>
@@ -132,6 +132,12 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -569,7 +575,10 @@
       </c>
       <c r="C8" s="4" t="inlineStr">
         <is>
-          <t>Classroom cum workshop – 500 - 600 sft (50-55 sqm)</t>
+          <t>Classroom – 350 sft (33 sqm)
+lab size – 500 sft (47 sqm)
+OR
+Classroom cum workshop – 500 sft (47 sqm)</t>
         </is>
       </c>
       <c r="D8" s="11" t="n"/>
@@ -634,13 +643,13 @@
       </c>
     </row>
     <row r="16" ht="14.15" customHeight="1">
-      <c r="A16" s="7" t="n">
+      <c r="A16" s="14" t="n">
         <v>1</v>
       </c>
       <c r="B16" s="8" t="inlineStr">
         <is>
-          <t>Laptop/ Desktop (Minimum Intel core i5-i3 6 gen or AMD Ryzen 5), Ram: minimum 8 - 16 GB, Graphic Card: dedicated GPU 2GB, High Speed Internet (Minimum 10 Mbps), Graphic Design Software 
-(Photoshop CC, Illustrator CC, CorelDraw)</t>
+          <t>Laptop/ Desktop (Minimum Intel core i5 or Intel core i3 6 gen/above, or AMD Ryzen 5/ similar spec; Ram: minimum 8 - 16 GB; Display: FHD monitor; Graphic Card: dedicated GPU 2GB; High Speed Internet (Minimum 10 Mbps); Graphic Design Software 
+(Photoshop CC, Illustrator CC, InDesign, After Effects, CorelDraw); 3D Design Software (Blender, Cinema 4D or Autodesk Maya)</t>
         </is>
       </c>
       <c r="C16" s="9" t="n">
@@ -659,7 +668,7 @@
       <c r="G16" s="9" t="n"/>
     </row>
     <row r="17" ht="14.15" customHeight="1">
-      <c r="A17" s="7" t="n">
+      <c r="A17" s="14" t="n">
         <v>2</v>
       </c>
       <c r="B17" s="8" t="inlineStr">
@@ -683,7 +692,7 @@
       <c r="G17" s="9" t="n"/>
     </row>
     <row r="18" ht="14.15" customHeight="1">
-      <c r="A18" s="7" t="n">
+      <c r="A18" s="14" t="n">
         <v>3</v>
       </c>
       <c r="B18" s="8" t="inlineStr">
@@ -707,7 +716,7 @@
       <c r="G18" s="9" t="n"/>
     </row>
     <row r="19" ht="14.15" customHeight="1">
-      <c r="A19" s="7" t="n">
+      <c r="A19" s="14" t="n">
         <v>4</v>
       </c>
       <c r="B19" s="8" t="inlineStr">
@@ -731,7 +740,7 @@
       <c r="G19" s="9" t="n"/>
     </row>
     <row r="20" ht="14.15" customHeight="1">
-      <c r="A20" s="7" t="n">
+      <c r="A20" s="14" t="n">
         <v>5</v>
       </c>
       <c r="B20" s="8" t="inlineStr">
@@ -755,7 +764,7 @@
       <c r="G20" s="9" t="n"/>
     </row>
     <row r="21" ht="14.15" customHeight="1">
-      <c r="A21" s="7" t="n">
+      <c r="A21" s="14" t="n">
         <v>6</v>
       </c>
       <c r="B21" s="8" t="inlineStr">
@@ -779,7 +788,7 @@
       <c r="G21" s="9" t="n"/>
     </row>
     <row r="22" ht="14.15" customHeight="1">
-      <c r="A22" s="7" t="n">
+      <c r="A22" s="14" t="n">
         <v>7</v>
       </c>
       <c r="B22" s="8" t="inlineStr">
@@ -803,16 +812,16 @@
       <c r="G22" s="9" t="n"/>
     </row>
     <row r="23" ht="14.15" customHeight="1">
-      <c r="A23" s="7" t="n">
+      <c r="A23" s="14" t="n">
         <v>8</v>
       </c>
       <c r="B23" s="8" t="inlineStr">
         <is>
-          <t>Air-conditioning (suited with workshop lab size)</t>
+          <t>Ergonomic chairs and desks (Plastic chairs/stool not acceptable)</t>
         </is>
       </c>
       <c r="C23" s="9" t="n">
-        <v>1</v>
+        <v>26</v>
       </c>
       <c r="D23" s="9" t="n">
         <v>0</v>
@@ -826,96 +835,80 @@
       </c>
       <c r="G23" s="9" t="n"/>
     </row>
-    <row r="24" ht="14.15" customHeight="1">
-      <c r="A24" s="7" t="n">
-        <v>9</v>
-      </c>
-      <c r="B24" s="8" t="inlineStr">
-        <is>
-          <t>Ergonomic chairs and desks (Plastic chairs/stool not acceptable)</t>
-        </is>
-      </c>
-      <c r="C24" s="9" t="n">
-        <v>26</v>
-      </c>
-      <c r="D24" s="9" t="n">
-        <v>0</v>
-      </c>
-      <c r="E24" s="9" t="n">
-        <v>5</v>
-      </c>
-      <c r="F24" s="9">
-        <f>IFERROR(MIN(C24,D24)*E24/C24,0)</f>
-        <v/>
-      </c>
-      <c r="G24" s="9" t="n"/>
+    <row r="24">
+      <c r="A24" s="15" t="inlineStr">
+        <is>
+          <t>Sum</t>
+        </is>
+      </c>
+      <c r="B24" s="11" t="n"/>
+      <c r="C24" s="11" t="n"/>
+      <c r="D24" s="12" t="n"/>
+      <c r="E24" s="15">
+        <f>SUM(E16:E23)</f>
+        <v/>
+      </c>
+      <c r="F24" s="15">
+        <f>SUM(F16:F23)</f>
+        <v/>
+      </c>
+      <c r="G24" s="13" t="n"/>
     </row>
     <row r="25">
-      <c r="A25" s="10" t="inlineStr">
-        <is>
-          <t>Sum</t>
+      <c r="A25" s="15" t="inlineStr">
+        <is>
+          <t>Score out of 100</t>
         </is>
       </c>
       <c r="B25" s="11" t="n"/>
       <c r="C25" s="11" t="n"/>
-      <c r="D25" s="12" t="n"/>
-      <c r="E25" s="10">
-        <f>SUM(E16:E24)</f>
-        <v/>
-      </c>
-      <c r="F25" s="10">
-        <f>SUM(F16:F24)</f>
+      <c r="D25" s="11" t="n"/>
+      <c r="E25" s="12" t="n"/>
+      <c r="F25" s="15">
+        <f>F24/E24*100</f>
         <v/>
       </c>
       <c r="G25" s="13" t="n"/>
     </row>
-    <row r="26">
-      <c r="A26" s="10" t="inlineStr">
-        <is>
-          <t>Score out of 100</t>
-        </is>
-      </c>
-      <c r="B26" s="11" t="n"/>
-      <c r="C26" s="11" t="n"/>
-      <c r="D26" s="11" t="n"/>
-      <c r="E26" s="12" t="n"/>
-      <c r="F26" s="10">
-        <f>F25/E25*100</f>
-        <v/>
-      </c>
-      <c r="G26" s="13" t="n"/>
-    </row>
-    <row r="27" ht="9.75" customHeight="1"/>
-    <row r="28">
-      <c r="A28" s="10" t="inlineStr">
+    <row r="26" ht="9.75" customHeight="1"/>
+    <row r="27">
+      <c r="A27" s="15" t="inlineStr">
         <is>
           <t xml:space="preserve">Total achieved points out of 30  </t>
         </is>
       </c>
-      <c r="B28" s="11" t="n"/>
-      <c r="C28" s="11" t="n"/>
-      <c r="D28" s="11" t="n"/>
-      <c r="E28" s="12" t="n"/>
-      <c r="F28" s="10">
-        <f>F26*30/100</f>
-        <v/>
-      </c>
-      <c r="G28" s="10" t="inlineStr">
+      <c r="B27" s="11" t="n"/>
+      <c r="C27" s="11" t="n"/>
+      <c r="D27" s="11" t="n"/>
+      <c r="E27" s="12" t="n"/>
+      <c r="F27" s="15">
+        <f>F25*30/100</f>
+        <v/>
+      </c>
+      <c r="G27" s="15" t="inlineStr">
         <is>
           <t>Points</t>
         </is>
       </c>
     </row>
+    <row r="28" ht="14.15" customHeight="1">
+      <c r="A28" s="5" t="inlineStr">
+        <is>
+          <t>* For this course, the lab should be air-conditioned. Otherwise, the total points achieved will be halved.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <mergeCells count="8">
+  <mergeCells count="9">
     <mergeCell ref="A13:G13"/>
     <mergeCell ref="C7:G7"/>
     <mergeCell ref="A1:G1"/>
-    <mergeCell ref="A26:E26"/>
-    <mergeCell ref="A27:G27"/>
-    <mergeCell ref="A28:E28"/>
-    <mergeCell ref="A25:D25"/>
+    <mergeCell ref="A25:E25"/>
+    <mergeCell ref="A26:G26"/>
+    <mergeCell ref="A24:D24"/>
     <mergeCell ref="C8:G8"/>
+    <mergeCell ref="A27:E27"/>
+    <mergeCell ref="A28:G28"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>